<commit_message>
Update test screenshots and test data
</commit_message>
<xml_diff>
--- a/src/test/resources/DemoWebShop_TestData.xlsx
+++ b/src/test/resources/DemoWebShop_TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclispse\NewWorkspace\DemoWebShopProject\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\DemoWebShopProject (1)\DemoWebShopProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46E9980C-6014-478C-B831-B5D47C597F0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9538B223-CDFE-48D7-8420-A8BD6FE49C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SignupLoginData" sheetId="1" r:id="rId1"/>
@@ -138,12 +138,6 @@
     <t>TC-AUTH-06</t>
   </si>
   <si>
-    <t>appunayak176@gmail.com</t>
-  </si>
-  <si>
-    <t>appu@123</t>
-  </si>
-  <si>
     <t>TC-AUTH-08</t>
   </si>
   <si>
@@ -249,9 +243,6 @@
     <t>TC-LOGOUT-05</t>
   </si>
   <si>
-    <t>Appu Nayak</t>
-  </si>
-  <si>
     <t>Please contact me regarding a product.</t>
   </si>
   <si>
@@ -262,6 +253,15 @@
   </si>
   <si>
     <t>TC-CHK-10</t>
+  </si>
+  <si>
+    <t>bvishwa78@gmail.com</t>
+  </si>
+  <si>
+    <t>Vish@123</t>
+  </si>
+  <si>
+    <t>Vishwanath</t>
   </si>
 </sst>
 </file>
@@ -627,7 +627,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
@@ -637,7 +637,7 @@
     <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -660,7 +660,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -680,12 +680,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -708,45 +708,45 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>34</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>35</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
-      <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
         <v>32</v>
@@ -754,6 +754,13 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G7" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{FD3BB272-8E2B-4ED9-9750-605856D7B978}"/>
+    <hyperlink ref="C5" r:id="rId2" xr:uid="{C20984C4-1879-4218-8019-F06A1416644D}"/>
+    <hyperlink ref="B6" r:id="rId3" xr:uid="{940469CD-5F32-4C26-9303-B83BE8A7B74F}"/>
+    <hyperlink ref="B7" r:id="rId4" xr:uid="{979FEA10-A2B6-445E-8A27-6DAF101BA805}"/>
+    <hyperlink ref="C7" r:id="rId5" xr:uid="{B4B055B6-E738-44AE-AE79-E39CA029D8DA}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -761,50 +768,50 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>42</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>44</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>46</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -816,7 +823,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -825,7 +832,7 @@
     <col min="6" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -848,7 +855,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -859,7 +866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -870,7 +877,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -881,7 +888,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -892,7 +899,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -903,7 +910,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -914,7 +921,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -934,7 +941,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
@@ -945,7 +952,7 @@
     <col min="10" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -959,7 +966,7 @@
         <v>18</v>
       </c>
       <c r="E1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -968,24 +975,24 @@
         <v>5</v>
       </c>
       <c r="H1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" t="s">
         <v>51</v>
-      </c>
-      <c r="I1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J1" t="s">
-        <v>53</v>
       </c>
       <c r="K1" t="s">
         <v>6</v>
       </c>
       <c r="L1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -994,30 +1001,30 @@
         <v>27</v>
       </c>
       <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" t="s">
         <v>56</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>57</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>58</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>59</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>60</v>
       </c>
-      <c r="K2" t="s">
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>61</v>
-      </c>
-      <c r="L2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>63</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -1026,30 +1033,30 @@
         <v>27</v>
       </c>
       <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" t="s">
         <v>56</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>57</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>58</v>
       </c>
-      <c r="H3" t="s">
+      <c r="K3" t="s">
         <v>59</v>
       </c>
-      <c r="I3" t="s">
+      <c r="L3" t="s">
         <v>60</v>
       </c>
-      <c r="K3" t="s">
-        <v>61</v>
-      </c>
-      <c r="L3" t="s">
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>64</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -1058,30 +1065,30 @@
         <v>27</v>
       </c>
       <c r="D4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" t="s">
         <v>56</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>57</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>58</v>
       </c>
-      <c r="H4" t="s">
+      <c r="K4" t="s">
         <v>59</v>
       </c>
-      <c r="I4" t="s">
+      <c r="L4" t="s">
         <v>60</v>
       </c>
-      <c r="K4" t="s">
-        <v>61</v>
-      </c>
-      <c r="L4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -1090,35 +1097,35 @@
         <v>27</v>
       </c>
       <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" t="s">
         <v>56</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>57</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>58</v>
       </c>
-      <c r="H5" t="s">
+      <c r="K5" t="s">
         <v>59</v>
       </c>
-      <c r="I5" t="s">
+      <c r="L5" t="s">
         <v>60</v>
       </c>
-      <c r="K5" t="s">
-        <v>61</v>
-      </c>
-      <c r="L5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B7" t="s">
         <v>33</v>
@@ -1130,27 +1137,27 @@
         <v>31</v>
       </c>
       <c r="F7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" t="s">
         <v>57</v>
       </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>58</v>
       </c>
-      <c r="H7" t="s">
+      <c r="K7" t="s">
         <v>59</v>
       </c>
-      <c r="I7" t="s">
+      <c r="L7" t="s">
         <v>60</v>
       </c>
-      <c r="K7" t="s">
-        <v>61</v>
-      </c>
-      <c r="L7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
         <v>33</v>
@@ -1159,30 +1166,30 @@
         <v>27</v>
       </c>
       <c r="D8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" t="s">
         <v>56</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
         <v>58</v>
       </c>
-      <c r="H8" t="s">
+      <c r="K8" t="s">
         <v>59</v>
       </c>
-      <c r="I8" t="s">
+      <c r="L8" t="s">
         <v>60</v>
       </c>
-      <c r="K8" t="s">
-        <v>61</v>
-      </c>
-      <c r="L8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
         <v>33</v>
@@ -1191,19 +1198,19 @@
         <v>27</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="F9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" t="s">
         <v>57</v>
       </c>
-      <c r="G9" t="s">
+      <c r="I9" t="s">
         <v>58</v>
-      </c>
-      <c r="H9" t="s">
-        <v>59</v>
-      </c>
-      <c r="I9" t="s">
-        <v>60</v>
       </c>
       <c r="K9">
         <v>90001</v>
@@ -1224,7 +1231,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1233,51 +1240,54 @@
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C1" t="s">
         <v>18</v>
       </c>
       <c r="D1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>71</v>
       </c>
-      <c r="B2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>74</v>
-      </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="28.75" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="A1:E16" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{613A7718-DF57-4DDF-9215-059D3A33A95F}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>